<commit_message>
refactor: archive legacy drafts and walkthrough notes while updating core thesis documentation and results
</commit_message>
<xml_diff>
--- a/results/02_4tier_filtering/02_4tier_filtering.xlsx
+++ b/results/02_4tier_filtering/02_4tier_filtering.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Table_of_Contents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Section_2A_Four_Tiered_Purposiv" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Section_2B_Nine_Airport_Experim" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Table_C_Summary_Descriptive_Sta" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Table_D_Filtered_9_Airports_Ind" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_of_Contents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section_2A_Four_Tiered_Purposiv" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Section_2B_Nine_Airport_Experim" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_C_Summary_Descriptive_Sta" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table_D_Filtered_9_Airports_Ind" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Section_2A_Four_Tiered_Purposiv'!$A$1:$F$5</definedName>
@@ -802,7 +802,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Collapses carrier collinearity (r&gt;=0.88; kappa&gt;10^4) to orthogonal Wiener-Hopf deconvolution (P(j*|k)=1.0)</t>
+          <t>Collapses carrier collinearity (r&gt;=0.88; kappa&gt;10^4) to single-carrier checkpoint isolation (P(j*|k)=1.0)</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2291,7 @@
       </c>
       <c r="S2" s="6" t="inlineStr">
         <is>
-          <t>Type I: Hard Physical Exclusivity (Air-Gapped Sterile Area)</t>
+          <t>Physically Separate Terminals (Air-Gapped Sterile Area)</t>
         </is>
       </c>
       <c r="T2" s="6" t="inlineStr">
@@ -2383,7 +2383,7 @@
       </c>
       <c r="S3" s="6" t="inlineStr">
         <is>
-          <t>Type II: Operational Exclusivity (Curbside/Ticketing Dedicated with Airside APM)</t>
+          <t>Walkway-Connected Terminals (Curbside/Ticketing Dedicated with Airside APM)</t>
         </is>
       </c>
       <c r="T3" s="6" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="S4" s="6" t="inlineStr">
         <is>
-          <t>Type I: Hard Physical Exclusivity (Air-Gapped Sterile Area)</t>
+          <t>Physically Separate Terminals (Air-Gapped Sterile Area)</t>
         </is>
       </c>
       <c r="T4" s="6" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
-          <t>Type I: Hard Physical Exclusivity (Air-Gapped Sterile Area)</t>
+          <t>Physically Separate Terminals (Air-Gapped Sterile Area)</t>
         </is>
       </c>
       <c r="T5" s="6" t="inlineStr">
@@ -2659,7 +2659,7 @@
       </c>
       <c r="S6" s="6" t="inlineStr">
         <is>
-          <t>Type II: Operational Exclusivity (Curbside/Ticketing Dedicated with Airside APM)</t>
+          <t>Walkway-Connected Terminals (Curbside/Ticketing Dedicated with Airside APM)</t>
         </is>
       </c>
       <c r="T6" s="6" t="inlineStr">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="S7" s="6" t="inlineStr">
         <is>
-          <t>Type II: Operational Exclusivity (Landside-Dedicated with Airside Pedestrian Connectors)</t>
+          <t>Walkway-Connected Terminals (Landside-Dedicated with Airside Pedestrian Connectors)</t>
         </is>
       </c>
       <c r="T7" s="6" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="S8" s="6" t="inlineStr">
         <is>
-          <t>Type I: Hard Physical Exclusivity (Air-Gapped Sterile Area)</t>
+          <t>Physically Separate Terminals (Air-Gapped Sterile Area)</t>
         </is>
       </c>
       <c r="T8" s="6" t="inlineStr">
@@ -2935,7 +2935,7 @@
       </c>
       <c r="S9" s="6" t="inlineStr">
         <is>
-          <t>Type I: Hard Physical Exclusivity (Air-Gapped Sterile Area)</t>
+          <t>Physically Separate Terminals (Air-Gapped Sterile Area)</t>
         </is>
       </c>
       <c r="T9" s="6" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="S10" s="6" t="inlineStr">
         <is>
-          <t>Type II: Operational Exclusivity (Curbside/Ticketing Dedicated with Airside Pedestrian Walkway)</t>
+          <t>Walkway-Connected Terminals (Curbside/Ticketing Dedicated with Airside Pedestrian Walkway)</t>
         </is>
       </c>
       <c r="T10" s="6" t="inlineStr">

</xml_diff>